<commit_message>
Add .gitattributes file for G-code documentation and update feathergauge part list
</commit_message>
<xml_diff>
--- a/build_info/Feather v4 Build List.xlsx
+++ b/build_info/Feather v4 Build List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bretwebb/Desktop/Currently Working On/USCRP Barrier Island Extreme Events/gage build/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hw_projects\feathergauge\build_info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC21755C-5AF1-3941-B77D-598A3695ADF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D4F6D8-6F5A-4CF7-918C-F361E7C3D1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1260" yWindow="760" windowWidth="28300" windowHeight="18540" xr2:uid="{235735D9-301C-4B49-97BC-5253FAC724FB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{235735D9-301C-4B49-97BC-5253FAC724FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,12 +107,6 @@
     <t>CR1220 12mm Diameter Coin Cell Battery</t>
   </si>
   <si>
-    <t>https://bluerobotics.com/store/sensors-cameras/sensors/bar02-sensor-r1-rp/</t>
-  </si>
-  <si>
-    <t>Bar02 Ultra High Resolution 10m Depth/Pressure Sensor</t>
-  </si>
-  <si>
     <t>1.5" PVC Pipe</t>
   </si>
   <si>
@@ -183,6 +177,12 @@
   </si>
   <si>
     <t>https://www.amazon.com/dp/B01M7V19JE?ref=fed_asin_title&amp;th=1</t>
+  </si>
+  <si>
+    <t>https://www.sparkfun.com/sparkfun-pressure-sensor-breakout-ms5803-14ba.html</t>
+  </si>
+  <si>
+    <t>SparkFun Pressure Sensor Breakout - MS5803-14BA</t>
   </si>
 </sst>
 </file>
@@ -615,20 +615,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D81BD6B-69B9-BB4B-8D95-67B130ED7761}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" customWidth="1"/>
-    <col min="2" max="2" width="65.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="111.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.3125" customWidth="1"/>
+    <col min="2" max="2" width="65.6875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.3125" customWidth="1"/>
+    <col min="6" max="6" width="111.1875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
@@ -648,7 +648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -669,7 +669,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="4">
         <f>A5+1</f>
         <v>2</v>
@@ -691,7 +691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="4">
         <f t="shared" ref="A7:A24" si="1">A6+1</f>
         <v>3</v>
@@ -713,7 +713,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="4">
         <f t="shared" si="1"/>
         <v>4</v>
@@ -735,7 +735,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="4">
         <f t="shared" si="1"/>
         <v>5</v>
@@ -757,7 +757,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="4">
         <f t="shared" si="1"/>
         <v>6</v>
@@ -779,7 +779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="4">
         <f t="shared" si="1"/>
         <v>7</v>
@@ -801,7 +801,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="4">
         <f t="shared" si="1"/>
         <v>8</v>
@@ -823,35 +823,35 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="4">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="C13" s="3">
-        <v>75</v>
+        <v>80.5</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" s="2">
         <f t="shared" si="0"/>
-        <v>75</v>
+        <v>80.5</v>
       </c>
       <c r="F13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A14" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
       </c>
       <c r="C14" s="3">
         <f>10.86/5</f>
@@ -866,16 +866,16 @@
         <v>1.4479999999999997</v>
       </c>
       <c r="F14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A15" s="4">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="4">
-        <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-      <c r="B15" t="s">
-        <v>28</v>
       </c>
       <c r="C15" s="3">
         <v>2.29</v>
@@ -888,16 +888,16 @@
         <v>2.29</v>
       </c>
       <c r="F15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="4">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C16" s="3">
         <v>1.69</v>
@@ -910,16 +910,16 @@
         <v>1.69</v>
       </c>
       <c r="F16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A17" s="4">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" s="3">
         <v>5.65</v>
@@ -932,16 +932,16 @@
         <v>5.65</v>
       </c>
       <c r="F17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A18" s="4">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-      <c r="B18" t="s">
-        <v>33</v>
       </c>
       <c r="C18" s="3">
         <v>11.68</v>
@@ -954,16 +954,16 @@
         <v>0.1168</v>
       </c>
       <c r="F18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C19" s="3">
         <v>6.48</v>
@@ -976,16 +976,16 @@
         <v>0.32400000000000007</v>
       </c>
       <c r="F19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="4">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C20" s="3">
         <f>4.29/12</f>
@@ -999,16 +999,16 @@
         <v>0.35749999999999998</v>
       </c>
       <c r="F20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="4">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C21" s="3">
         <f>9.31/50</f>
@@ -1022,16 +1022,16 @@
         <v>0.74480000000000002</v>
       </c>
       <c r="F21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="4">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C22" s="3">
         <f>6.14/100</f>
@@ -1045,16 +1045,16 @@
         <v>0.24559999999999998</v>
       </c>
       <c r="F22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A23" s="4">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="B23" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="4">
-        <f t="shared" si="1"/>
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>43</v>
       </c>
       <c r="C23" s="3">
         <v>0</v>
@@ -1067,16 +1067,16 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="7">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C24" s="9">
         <v>0</v>
@@ -1089,21 +1089,21 @@
         <v>0</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="E25" s="2">
         <f>SUM(E5:E24)</f>
-        <v>162.76670000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+        <v>168.26670000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C27" s="3">
         <f>9.99/60</f>
@@ -1117,7 +1117,7 @@
         <v>0.16650000000000001</v>
       </c>
       <c r="F27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>